<commit_message>
Fix MULNV name, add novelty triage helper
- Index/ministerien.xlsx: MULNV name war "Ministerium für Umwelt,
  Landwirtschaft, Naturschutz und Verkehr" — falscher Ressortzuschnitt.
  Korrekter WP17-Name: "...Natur- und Verbraucherschutz". Bug erklärt
  ~1400 von 1632 ministerium_form-Einträgen in vocab_novelty.log
  (Token-Match auf MLV statt MULNV bei Containment 0.50).

- build_novelty_table.py: Aggregiert ministerium_form-Einträge aus
  data/vocab_novelty.log nach data/ministerium_novelty.xlsx, mit
  Vorschlag-Kürzel (top Containment / Jaccard) für Operator-Triage.

- .gitignore: LibreOffice .~lock-Files.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Index/ministerien.xlsx
+++ b/Index/ministerien.xlsx
@@ -16958,7 +16958,7 @@
       </c>
       <c r="B16" s="9" t="inlineStr">
         <is>
-          <t>Ministerium für Umwelt, Landwirtschaft, Naturschutz und Verkehr</t>
+          <t>Ministerium für Umwelt, Landwirtschaft, Natur- und Verbraucherschutz</t>
         </is>
       </c>
       <c r="D16" s="5" t="n">
@@ -17056,12 +17056,12 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
+      <c r="A22" s="7" t="inlineStr">
         <is>
           <t>MP</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="B22" s="7" t="inlineStr">
         <is>
           <t>Ministerpräsident</t>
         </is>
@@ -17310,13 +17310,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A829E164-467C-49DC-B787-47889157C1BD}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{66877F6F-D922-4929-8512-2648396A7324}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AEFFDEA5-51B7-4173-AC0C-D88B359192BE}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6F92FC2D-E9A9-47D7-BFAE-739447CF0914}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2D796116-370E-4F8A-BB61-290D92C084EB}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9729EA6E-CCB9-477B-9F6B-D261B32188F7}"/>
 </file>
</xml_diff>